<commit_message>
Restyle the workbook and templates to the repository's Mermaid palette
Titles, links and function cells move to Tyrian purple; inputs to platinum; header labels and text on dark fills to ivory; warnings and the TOC length guard to crimson; passed checks in the cash-flow template to Rhodesian green. Tabs and theme colours follow the same roles. Only formatting changes: no formula, value or cached result moves. workbook_palette.py applies the palette, with --template for templates/.
</commit_message>
<xml_diff>
--- a/templates/13-week-cash-flow-forecast.xlsx
+++ b/templates/13-week-cash-flow-forecast.xlsx
@@ -83,31 +83,31 @@
     <x:numFmt numFmtId="203" formatCode="0"/>
     <x:numFmt numFmtId="204" formatCode="#,##0;[Red](#,##0);-"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF2B2733"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="18"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:color rgb="FFFFFFF0"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="FF2B2733"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:color rgb="FFFFFFF0"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -127,24 +127,24 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FFC00000"/>
+      <x:color rgb="FF990024"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF4F485E"/>
+      <x:color rgb="FF66023C"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF2B2733"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF04001F"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -156,11 +156,16 @@
     <x:font>
       <x:b/>
       <x:sz val="12"/>
-      <x:color rgb="FF04001F"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0F4B32"/>
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
@@ -173,47 +178,47 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF5C2D91"/>
+        <x:fgColor rgb="FF66023C"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF3F1F6"/>
+        <x:fgColor rgb="FFFFFFF0"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFC00000"/>
+        <x:fgColor rgb="FF990024"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF04001F"/>
+        <x:fgColor rgb="FF000000"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFCE4D6"/>
+        <x:fgColor rgb="FFF0D9DE"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE2F0D9"/>
+        <x:fgColor rgb="FFDBE4E0"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF7A5AB5"/>
+        <x:fgColor rgb="FF990024"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDED9E8"/>
+        <x:fgColor rgb="FFE8D9E2"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFB1AFAD"/>
+        <x:fgColor rgb="FFE5E4E2"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -226,7 +231,7 @@
     <x:border/>
     <x:border>
       <x:bottom style="double">
-        <x:color rgb="FF4F485E"/>
+        <x:color rgb="FF66023C"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -264,7 +269,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -381,364 +386,364 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF5C2D91"/>
+        <x:color rgb="FF66023C"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDED9E8"/>
+          <x:bgColor rgb="FFE8D9E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF5C2D91"/>
+        <x:color rgb="FF66023C"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDED9E8"/>
+          <x:bgColor rgb="FFE8D9E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF5C2D91"/>
+        <x:color rgb="FF66023C"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDED9E8"/>
+          <x:bgColor rgb="FFE8D9E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF5C2D91"/>
+        <x:color rgb="FF66023C"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDED9E8"/>
+          <x:bgColor rgb="FFE8D9E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF5C2D91"/>
+        <x:color rgb="FF66023C"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDED9E8"/>
+          <x:bgColor rgb="FFE8D9E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF008000"/>
+        <x:color rgb="FF0F4B32"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
+          <x:bgColor rgb="FFDBE4E0"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF990024"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFF0D9DE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF5C2D91"/>
+        <x:color rgb="FF66023C"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDED9E8"/>
+          <x:bgColor rgb="FFE8D9E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1170,34 +1175,34 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="F3F1F6"/>
+        <a:srgbClr val="FFFFF0"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5C2D91"/>
+        <a:srgbClr val="66023C"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="04001F"/>
+        <a:srgbClr val="990024"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="7A5AB5"/>
+        <a:srgbClr val="E5E4E2"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="4F485E"/>
+        <a:srgbClr val="6E6862"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="DED9E8"/>
+        <a:srgbClr val="B1AFAD"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="B1AFAD"/>
+        <a:srgbClr val="DCDAD7"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="7A5AB5"/>
+        <a:srgbClr val="66023C"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="4F485E"/>
+        <a:srgbClr val="990024"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1696,7 +1701,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="17" t="str">
-        <x:v>Blue text / lavender fill</x:v>
+        <x:v>Blue text / ivory fill</x:v>
       </x:c>
       <x:c r="B24" s="75" t="str">
         <x:v>Editable user input</x:v>

</xml_diff>